<commit_message>
Deployed bff4fef with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/asset/แบบฟอร์ม สมอ.1.xlsx
+++ b/asset/แบบฟอร์ม สมอ.1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\วิทยาลัย\เทคนิคสุพรรณบุรี\งานอาคารวิทยบริการและห้องสมุด\งานซื้อหนังสือ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krube\my-project\docs\asset\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -137,13 +137,13 @@
     <t>รหัสวิชา.............................................. ชื่อวิชา...................................................................... ระดับชั้น......... ครูผู้สอน........................................................</t>
   </si>
   <si>
-    <t>ลงชื่อ.........................................................ครูผู้สอน                ลงชื่อ.........................................................ครูผู้สอน                 ลงชื่อ.........................................................ครูผู้สอน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">                                                                         (......................................................)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      (.......................................................)                                (.........................................................)                                 (.........................................................)     </t>
+    <t>ลงชื่อ.........................................................ครูผู้สอน            ลงชื่อ.........................................................ครูผู้สอน          ลงชื่อ.........................................................ครูผู้สอน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      (.......................................................)                           (.........................................................)                         (.........................................................)     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                                                             (......................................................)</t>
   </si>
 </sst>
 </file>
@@ -287,9 +287,15 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -301,12 +307,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -640,168 +640,169 @@
     <col min="14" max="14" width="5.19921875" customWidth="1"/>
     <col min="15" max="15" width="5.69921875" customWidth="1"/>
     <col min="16" max="16" width="7.8984375" customWidth="1"/>
+    <col min="17" max="17" width="14.796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
     </row>
     <row r="3" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="15"/>
     </row>
     <row r="4" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
     </row>
     <row r="5" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="13"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
     </row>
     <row r="6" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
     </row>
     <row r="8" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="14" t="s">
+      <c r="C8" s="17"/>
+      <c r="D8" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14" t="s">
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14" t="s">
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14" t="s">
+      <c r="M8" s="16"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="P8" s="14" t="s">
+      <c r="P8" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="Q8" s="14" t="s">
+      <c r="Q8" s="16" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="42" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="16"/>
       <c r="B9" s="8" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
       <c r="F9" s="10" t="s">
         <v>15</v>
       </c>
@@ -829,9 +830,9 @@
       <c r="N9" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="O9" s="14"/>
-      <c r="P9" s="14"/>
-      <c r="Q9" s="14"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+      <c r="Q9" s="16"/>
     </row>
     <row r="10" spans="1:17" ht="21" x14ac:dyDescent="0.25">
       <c r="A10" s="6">
@@ -900,144 +901,139 @@
       <c r="A13" s="4"/>
     </row>
     <row r="14" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="16"/>
-      <c r="O14" s="16"/>
-      <c r="P14" s="16"/>
-      <c r="Q14" s="16"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="11"/>
     </row>
     <row r="15" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="11"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="12"/>
     </row>
     <row r="16" spans="1:17" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
     </row>
     <row r="17" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="11"/>
-      <c r="Q17" s="11"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+      <c r="P17" s="12"/>
+      <c r="Q17" s="12"/>
     </row>
     <row r="18" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="11"/>
-      <c r="P18" s="11"/>
-      <c r="Q18" s="11"/>
+      <c r="A18" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="12"/>
     </row>
     <row r="19" spans="1:17" ht="21" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
     </row>
     <row r="20" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="17"/>
-      <c r="O20" s="17"/>
-      <c r="P20" s="17"/>
-      <c r="Q20" s="17"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
+      <c r="P20" s="13"/>
+      <c r="Q20" s="13"/>
     </row>
     <row r="21" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A21" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="11"/>
+      <c r="A21" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="12"/>
+      <c r="P21" s="12"/>
+      <c r="Q21" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A14:Q14"/>
-    <mergeCell ref="A15:Q15"/>
-    <mergeCell ref="A17:Q17"/>
-    <mergeCell ref="A18:Q18"/>
-    <mergeCell ref="A20:Q20"/>
     <mergeCell ref="A21:Q21"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A3:Q3"/>
@@ -1054,8 +1050,13 @@
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="I8:K8"/>
     <mergeCell ref="L8:N8"/>
+    <mergeCell ref="A14:Q14"/>
+    <mergeCell ref="A15:Q15"/>
+    <mergeCell ref="A17:Q17"/>
+    <mergeCell ref="A18:Q18"/>
+    <mergeCell ref="A20:Q20"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.59055118110236227" right="0.39370078740157483" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>